<commit_message>
Fixed Council Tax file to include 10 areas
</commit_message>
<xml_diff>
--- a/Raw/Council Tax.xlsx
+++ b/Raw/Council Tax.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jabegu\Desktop\SQL\Principles-of-Data-Science-Coursework\Raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F9249FA2-14DA-4BBA-BAB1-AA6BB125B5FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A06BCB2-9592-41E7-9CFE-EEC9C46BC8A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{AAC90F36-24F6-4065-9BB2-86FA5D184E6E}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
   <si>
     <t>Area name</t>
   </si>
@@ -90,6 +90,9 @@
   </si>
   <si>
     <t>Wroxton</t>
+  </si>
+  <si>
+    <t>Launton</t>
   </si>
 </sst>
 </file>
@@ -462,7 +465,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EF279557-D1C5-4E82-8C4F-D58DC1D8B355}">
-  <dimension ref="A1:I10"/>
+  <dimension ref="A1:I11"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="9.6640625" bestFit="1" customWidth="1"/>
@@ -702,59 +705,88 @@
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="B9" s="1">
-        <v>1586.67</v>
+        <v>1624.26</v>
       </c>
       <c r="C9" s="1">
-        <v>1851.11</v>
+        <v>1894.96</v>
       </c>
       <c r="D9" s="1">
-        <v>2115.5500000000002</v>
+        <v>2165.67</v>
       </c>
       <c r="E9" s="1">
-        <v>2380</v>
+        <v>2436.38</v>
       </c>
       <c r="F9" s="1">
-        <v>2908.89</v>
+        <v>2977.8</v>
       </c>
       <c r="G9" s="1">
-        <v>3437.77</v>
+        <v>3519.21</v>
       </c>
       <c r="H9" s="1">
-        <v>3966.67</v>
+        <v>4060.64</v>
       </c>
       <c r="I9" s="1">
-        <v>4760</v>
+        <v>4872.76</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
+        <v>16</v>
+      </c>
+      <c r="B10" s="1">
+        <v>1586.67</v>
+      </c>
+      <c r="C10" s="1">
+        <v>1851.11</v>
+      </c>
+      <c r="D10" s="1">
+        <v>2115.5500000000002</v>
+      </c>
+      <c r="E10" s="1">
+        <v>2380</v>
+      </c>
+      <c r="F10" s="1">
+        <v>2908.89</v>
+      </c>
+      <c r="G10" s="1">
+        <v>3437.77</v>
+      </c>
+      <c r="H10" s="1">
+        <v>3966.67</v>
+      </c>
+      <c r="I10" s="1">
+        <v>4760</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
         <v>17</v>
       </c>
-      <c r="B10" s="1">
+      <c r="B11" s="1">
         <v>1592.13</v>
       </c>
-      <c r="C10" s="1">
+      <c r="C11" s="1">
         <v>1857.48</v>
       </c>
-      <c r="D10" s="1">
+      <c r="D11" s="1">
         <v>2122.83</v>
       </c>
-      <c r="E10" s="1">
+      <c r="E11" s="1">
         <v>2388.19</v>
       </c>
-      <c r="F10" s="1">
+      <c r="F11" s="1">
         <v>2918.9</v>
       </c>
-      <c r="G10" s="1">
+      <c r="G11" s="1">
         <v>3449.6</v>
       </c>
-      <c r="H10" s="1">
+      <c r="H11" s="1">
         <v>3980.32</v>
       </c>
-      <c r="I10" s="1">
+      <c r="I11" s="1">
         <v>4776.38</v>
       </c>
     </row>

</xml_diff>